<commit_message>
Ajout et correction partie i,terface graphique
</commit_message>
<xml_diff>
--- a/data/raw/recap_pssm.xlsx
+++ b/data/raw/recap_pssm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30002"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SSU\Echanges\Prévention collective\PSSM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Rapport d'activité\Rapport d'activité 2025-2026\Stage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D8D950-D43E-4C6C-B5AA-BA3FC48E112B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE38DFA-9C2C-4DAE-BB23-6B24C537441E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="15480" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PSSM 2021" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="136">
   <si>
     <t xml:space="preserve">Formations PSSM 2021 </t>
   </si>
@@ -451,28 +451,31 @@
     <t>Total année univ</t>
   </si>
   <si>
+    <t>Date début</t>
+  </si>
+  <si>
+    <t>Date fin</t>
+  </si>
+  <si>
     <t>Formatrice/teur</t>
   </si>
   <si>
-    <t>1 et 2/10/25</t>
-  </si>
-  <si>
-    <t>aco</t>
-  </si>
-  <si>
-    <t>23 et 24/10/25</t>
-  </si>
-  <si>
-    <t>20 et 21/11/25</t>
-  </si>
-  <si>
-    <t>25 et 26/11/25</t>
-  </si>
-  <si>
-    <t>4 et 5/12/25</t>
-  </si>
-  <si>
-    <t>10 et 11/12/25</t>
+    <t>Etab</t>
+  </si>
+  <si>
+    <t>Nb</t>
+  </si>
+  <si>
+    <t>Institut agro</t>
+  </si>
+  <si>
+    <t>UA</t>
+  </si>
+  <si>
+    <t>ARIFTS</t>
+  </si>
+  <si>
+    <t>Personnels</t>
   </si>
 </sst>
 </file>
@@ -564,7 +567,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="41">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -983,88 +986,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -1081,10 +1002,25 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top style="medium">
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -1092,7 +1028,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1238,25 +1174,28 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1282,18 +1221,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1582,26 +1509,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
     <col min="2" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1"/>
-    <row r="3" spans="1:9" ht="32.25" thickBot="1">
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+    </row>
+    <row r="2" spans="1:9" ht="15" thickBot="1"/>
+    <row r="3" spans="1:9" ht="31.9" thickBot="1">
       <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
@@ -1611,17 +1538,17 @@
       <c r="C3" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="63" t="s">
+      <c r="D3" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="64"/>
+      <c r="E3" s="65"/>
       <c r="F3" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="65" t="s">
+      <c r="G3" s="66" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="66"/>
+      <c r="H3" s="67"/>
     </row>
     <row r="4" spans="1:9" ht="36" customHeight="1">
       <c r="A4" s="12" t="s">
@@ -1833,7 +1760,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E763145-36B3-454E-B83B-697300787AF0}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
   </cols>
@@ -2106,7 +2033,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K24"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="30.140625" customWidth="1"/>
     <col min="2" max="3" width="12.7109375" customWidth="1"/>
@@ -2114,7 +2041,7 @@
     <col min="5" max="7" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="31.5">
+    <row r="1" spans="1:11" ht="31.15">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
@@ -2501,15 +2428,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15.75">
+    <row r="21" spans="1:11" ht="15.6">
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" ht="15.75">
+    <row r="22" spans="1:11" ht="15.6">
       <c r="K22" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.75">
+    <row r="23" spans="1:11" ht="15.6">
       <c r="K23" s="2">
         <v>1</v>
       </c>
@@ -2529,12 +2456,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3576EB05-E927-4119-ADA6-EBB7AECECC46}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="31.5">
+    <row r="1" spans="1:8" ht="31.15">
       <c r="A1" s="37" t="s">
         <v>1</v>
       </c>
@@ -2555,7 +2482,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.75">
+    <row r="2" spans="1:8" ht="15.6">
       <c r="A2" s="1" t="s">
         <v>40</v>
       </c>
@@ -2573,7 +2500,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="34"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75">
+    <row r="3" spans="1:8" ht="15.6">
       <c r="A3" s="2" t="s">
         <v>41</v>
       </c>
@@ -2591,7 +2518,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="34"/>
     </row>
-    <row r="4" spans="1:8" ht="15.75">
+    <row r="4" spans="1:8" ht="15.6">
       <c r="A4" s="2" t="s">
         <v>43</v>
       </c>
@@ -2613,7 +2540,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="34"/>
     </row>
-    <row r="5" spans="1:8" ht="15.75">
+    <row r="5" spans="1:8" ht="15.6">
       <c r="A5" s="2" t="s">
         <v>45</v>
       </c>
@@ -2635,7 +2562,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="34"/>
     </row>
-    <row r="6" spans="1:8" ht="15.75">
+    <row r="6" spans="1:8" ht="15.6">
       <c r="A6" s="2" t="s">
         <v>47</v>
       </c>
@@ -2649,7 +2576,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="34"/>
     </row>
-    <row r="7" spans="1:8" ht="15.75">
+    <row r="7" spans="1:8" ht="15.6">
       <c r="A7" s="2" t="s">
         <v>48</v>
       </c>
@@ -2671,7 +2598,7 @@
       <c r="G7" s="2"/>
       <c r="H7" s="34"/>
     </row>
-    <row r="8" spans="1:8" ht="15.75">
+    <row r="8" spans="1:8" ht="15.6">
       <c r="A8" s="2" t="s">
         <v>49</v>
       </c>
@@ -2693,7 +2620,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="34"/>
     </row>
-    <row r="9" spans="1:8" ht="15.75">
+    <row r="9" spans="1:8" ht="15.6">
       <c r="A9" s="2" t="s">
         <v>52</v>
       </c>
@@ -2711,7 +2638,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" ht="15.75">
+    <row r="10" spans="1:8" ht="15.6">
       <c r="A10" s="1" t="s">
         <v>55</v>
       </c>
@@ -2729,7 +2656,7 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" ht="15.75">
+    <row r="11" spans="1:8" ht="15.6">
       <c r="A11" s="1" t="s">
         <v>58</v>
       </c>
@@ -2747,7 +2674,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8" ht="15.75">
+    <row r="12" spans="1:8" ht="15.6">
       <c r="A12" s="2" t="s">
         <v>59</v>
       </c>
@@ -2767,7 +2694,7 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:8" ht="15.75">
+    <row r="13" spans="1:8" ht="15.6">
       <c r="A13" s="2" t="s">
         <v>60</v>
       </c>
@@ -2785,7 +2712,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" ht="15.75">
+    <row r="14" spans="1:8" ht="15.6">
       <c r="A14" s="2" t="s">
         <v>61</v>
       </c>
@@ -2803,7 +2730,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" ht="15.75">
+    <row r="15" spans="1:8" ht="15.6">
       <c r="A15" s="2" t="s">
         <v>34</v>
       </c>
@@ -2821,7 +2748,7 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8" ht="15.75">
+    <row r="16" spans="1:8" ht="15.6">
       <c r="A16" s="2" t="s">
         <v>62</v>
       </c>
@@ -2843,7 +2770,7 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" ht="15.75">
+    <row r="17" spans="1:8" ht="15.6">
       <c r="A17" s="2" t="s">
         <v>63</v>
       </c>
@@ -2861,7 +2788,7 @@
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" ht="15.75">
+    <row r="18" spans="1:8" ht="15.6">
       <c r="A18" s="2" t="s">
         <v>64</v>
       </c>
@@ -2883,7 +2810,7 @@
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" ht="15.75">
+    <row r="19" spans="1:8" ht="15.6">
       <c r="A19" s="2" t="s">
         <v>65</v>
       </c>
@@ -2909,7 +2836,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.75">
+    <row r="20" spans="1:8" ht="15.6">
       <c r="A20" s="2" t="s">
         <v>67</v>
       </c>
@@ -2931,7 +2858,7 @@
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8" ht="15.75">
+    <row r="21" spans="1:8" ht="15.6">
       <c r="A21" s="2" t="s">
         <v>68</v>
       </c>
@@ -3057,7 +2984,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="24.42578125" customWidth="1"/>
     <col min="2" max="3" width="12.7109375" customWidth="1"/>
@@ -3075,17 +3002,17 @@
       <c r="C1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="67" t="s">
+      <c r="D1" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="68"/>
+      <c r="E1" s="69"/>
       <c r="F1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="69" t="s">
+      <c r="G1" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="70"/>
+      <c r="H1" s="71"/>
       <c r="I1" s="36" t="s">
         <v>69</v>
       </c>
@@ -3610,7 +3537,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="15.75">
+    <row r="25" spans="1:9" ht="15.6">
       <c r="A25" s="10"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
@@ -3620,7 +3547,7 @@
       <c r="G25" s="7"/>
       <c r="H25" s="8"/>
     </row>
-    <row r="26" spans="1:9" ht="15.75">
+    <row r="26" spans="1:9" ht="15.6">
       <c r="A26" s="16"/>
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
@@ -3630,7 +3557,7 @@
       <c r="G26" s="17"/>
       <c r="H26" s="18"/>
     </row>
-    <row r="27" spans="1:9" ht="15.75">
+    <row r="27" spans="1:9" ht="15.6">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
@@ -3640,7 +3567,7 @@
       <c r="G27" s="7"/>
       <c r="H27" s="8"/>
     </row>
-    <row r="28" spans="1:9" ht="15.75">
+    <row r="28" spans="1:9" ht="15.6">
       <c r="A28" s="16"/>
       <c r="B28" s="16"/>
       <c r="C28" s="16"/>
@@ -3650,7 +3577,7 @@
       <c r="G28" s="17"/>
       <c r="H28" s="18"/>
     </row>
-    <row r="29" spans="1:9" ht="15.75">
+    <row r="29" spans="1:9" ht="15.6">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
@@ -3674,12 +3601,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84266D67-9F1E-45AD-9E62-480BFC5CBE01}">
   <dimension ref="A1:K33"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" thickBot="1">
+    <row r="1" spans="1:9" ht="31.9" thickBot="1">
       <c r="A1" s="31" t="s">
         <v>1</v>
       </c>
@@ -3689,19 +3616,19 @@
       <c r="C1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="67" t="s">
+      <c r="D1" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="68"/>
+      <c r="E1" s="69"/>
       <c r="F1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="69" t="s">
+      <c r="G1" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="70"/>
-    </row>
-    <row r="2" spans="1:9" ht="15.75">
+      <c r="H1" s="71"/>
+    </row>
+    <row r="2" spans="1:9" ht="15.6">
       <c r="A2" s="12" t="s">
         <v>81</v>
       </c>
@@ -3718,7 +3645,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75">
+    <row r="3" spans="1:9" ht="15.6">
       <c r="A3" s="11" t="s">
         <v>82</v>
       </c>
@@ -3740,7 +3667,7 @@
       <c r="G3" s="7"/>
       <c r="H3" s="8"/>
     </row>
-    <row r="4" spans="1:9" ht="15.75">
+    <row r="4" spans="1:9" ht="15.6">
       <c r="A4" s="11"/>
       <c r="B4" s="10"/>
       <c r="C4" s="11"/>
@@ -3754,7 +3681,7 @@
       <c r="G4" s="7"/>
       <c r="H4" s="8"/>
     </row>
-    <row r="5" spans="1:9" ht="15.75">
+    <row r="5" spans="1:9" ht="15.6">
       <c r="A5" s="11" t="s">
         <v>83</v>
       </c>
@@ -3774,7 +3701,7 @@
       <c r="G5" s="7"/>
       <c r="H5" s="8"/>
     </row>
-    <row r="6" spans="1:9" ht="15.75">
+    <row r="6" spans="1:9" ht="15.6">
       <c r="A6" s="1"/>
       <c r="B6" s="12"/>
       <c r="C6" s="11"/>
@@ -3788,7 +3715,7 @@
       <c r="G6" s="7"/>
       <c r="H6" s="8"/>
     </row>
-    <row r="7" spans="1:9" ht="15.75">
+    <row r="7" spans="1:9" ht="15.6">
       <c r="A7" s="1" t="s">
         <v>85</v>
       </c>
@@ -3808,7 +3735,7 @@
       <c r="G7" s="7"/>
       <c r="H7" s="8"/>
     </row>
-    <row r="8" spans="1:9" ht="15.75">
+    <row r="8" spans="1:9" ht="15.6">
       <c r="A8" s="34"/>
       <c r="B8" s="10"/>
       <c r="C8" s="11"/>
@@ -3822,7 +3749,7 @@
       <c r="G8" s="7"/>
       <c r="H8" s="8"/>
     </row>
-    <row r="9" spans="1:9" ht="15.75">
+    <row r="9" spans="1:9" ht="15.6">
       <c r="A9" s="2" t="s">
         <v>86</v>
       </c>
@@ -3844,7 +3771,7 @@
       <c r="G9" s="7"/>
       <c r="H9" s="8"/>
     </row>
-    <row r="10" spans="1:9" ht="15.75">
+    <row r="10" spans="1:9" ht="15.6">
       <c r="A10" s="2"/>
       <c r="B10" s="12"/>
       <c r="C10" s="11"/>
@@ -3858,7 +3785,7 @@
       <c r="G10" s="7"/>
       <c r="H10" s="8"/>
     </row>
-    <row r="11" spans="1:9" ht="15.75">
+    <row r="11" spans="1:9" ht="15.6">
       <c r="A11" s="10" t="s">
         <v>88</v>
       </c>
@@ -3880,7 +3807,7 @@
       <c r="G11" s="7"/>
       <c r="H11" s="8"/>
     </row>
-    <row r="12" spans="1:9" ht="15.75">
+    <row r="12" spans="1:9" ht="15.6">
       <c r="A12" s="10"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -3894,7 +3821,7 @@
       <c r="G12" s="7"/>
       <c r="H12" s="8"/>
     </row>
-    <row r="13" spans="1:9" ht="15.75">
+    <row r="13" spans="1:9" ht="15.6">
       <c r="A13" s="16" t="s">
         <v>89</v>
       </c>
@@ -3916,7 +3843,7 @@
       <c r="G13" s="17"/>
       <c r="H13" s="18"/>
     </row>
-    <row r="14" spans="1:9" ht="15.75">
+    <row r="14" spans="1:9" ht="15.6">
       <c r="A14" s="10"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -3930,7 +3857,7 @@
       <c r="G14" s="7"/>
       <c r="H14" s="8"/>
     </row>
-    <row r="15" spans="1:9" ht="15.75">
+    <row r="15" spans="1:9" ht="15.6">
       <c r="A15" s="16" t="s">
         <v>90</v>
       </c>
@@ -3952,7 +3879,7 @@
       <c r="G15" s="17"/>
       <c r="H15" s="18"/>
     </row>
-    <row r="16" spans="1:9" ht="15.75">
+    <row r="16" spans="1:9" ht="15.6">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -3966,7 +3893,7 @@
       <c r="G16" s="7"/>
       <c r="H16" s="8"/>
     </row>
-    <row r="17" spans="1:8" ht="15.75">
+    <row r="17" spans="1:8" ht="15.6">
       <c r="A17" s="16" t="s">
         <v>91</v>
       </c>
@@ -3988,7 +3915,7 @@
       <c r="G17" s="17"/>
       <c r="H17" s="18"/>
     </row>
-    <row r="18" spans="1:8" ht="15.75">
+    <row r="18" spans="1:8" ht="15.6">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -4002,7 +3929,7 @@
       <c r="G18" s="7"/>
       <c r="H18" s="8"/>
     </row>
-    <row r="19" spans="1:8" ht="15.75">
+    <row r="19" spans="1:8" ht="15.6">
       <c r="A19" s="16" t="s">
         <v>92</v>
       </c>
@@ -4018,7 +3945,7 @@
       <c r="G19" s="17"/>
       <c r="H19" s="18"/>
     </row>
-    <row r="20" spans="1:8" ht="15.75">
+    <row r="20" spans="1:8" ht="15.6">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -4028,7 +3955,7 @@
       <c r="G20" s="7"/>
       <c r="H20" s="8"/>
     </row>
-    <row r="21" spans="1:8" ht="15.75">
+    <row r="21" spans="1:8" ht="15.6">
       <c r="A21" s="16" t="s">
         <v>93</v>
       </c>
@@ -4050,7 +3977,7 @@
       <c r="G21" s="17"/>
       <c r="H21" s="18"/>
     </row>
-    <row r="22" spans="1:8" ht="15.75">
+    <row r="22" spans="1:8" ht="15.6">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -4064,7 +3991,7 @@
       <c r="G22" s="7"/>
       <c r="H22" s="8"/>
     </row>
-    <row r="23" spans="1:8" ht="15.75">
+    <row r="23" spans="1:8" ht="15.6">
       <c r="A23" s="16" t="s">
         <v>94</v>
       </c>
@@ -4086,7 +4013,7 @@
       <c r="G23" s="17"/>
       <c r="H23" s="18"/>
     </row>
-    <row r="24" spans="1:8" ht="15.75">
+    <row r="24" spans="1:8" ht="15.6">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -4100,7 +4027,7 @@
       <c r="G24" s="7"/>
       <c r="H24" s="8"/>
     </row>
-    <row r="25" spans="1:8" ht="15.75">
+    <row r="25" spans="1:8" ht="15.6">
       <c r="A25" s="16" t="s">
         <v>95</v>
       </c>
@@ -4122,7 +4049,7 @@
       <c r="G25" s="34"/>
       <c r="H25" s="34"/>
     </row>
-    <row r="26" spans="1:8" ht="15.75">
+    <row r="26" spans="1:8" ht="15.6">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -4165,12 +4092,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A84AC3-8203-45F5-A05D-F6156682D6EC}">
   <dimension ref="A1:I37"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" thickBot="1">
+    <row r="1" spans="1:9" ht="31.9" thickBot="1">
       <c r="A1" s="31" t="s">
         <v>1</v>
       </c>
@@ -4180,22 +4107,22 @@
       <c r="C1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="67" t="s">
+      <c r="D1" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="68"/>
+      <c r="E1" s="69"/>
       <c r="F1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="69" t="s">
+      <c r="G1" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="70"/>
+      <c r="H1" s="71"/>
       <c r="I1" s="36" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75">
+    <row r="2" spans="1:9" ht="15.6">
       <c r="A2" s="16" t="s">
         <v>70</v>
       </c>
@@ -4216,7 +4143,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75">
+    <row r="3" spans="1:9" ht="15.6">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -4241,7 +4168,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75">
+    <row r="4" spans="1:9" ht="15.6">
       <c r="A4" s="16" t="s">
         <v>73</v>
       </c>
@@ -4264,7 +4191,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75">
+    <row r="5" spans="1:9" ht="15.6">
       <c r="A5" s="16"/>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
@@ -4278,7 +4205,7 @@
       <c r="G5" s="17"/>
       <c r="H5" s="18"/>
     </row>
-    <row r="6" spans="1:9" ht="15.75">
+    <row r="6" spans="1:9" ht="15.6">
       <c r="A6" s="16"/>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
@@ -4292,7 +4219,7 @@
       <c r="G6" s="17"/>
       <c r="H6" s="18"/>
     </row>
-    <row r="7" spans="1:9" ht="15.75">
+    <row r="7" spans="1:9" ht="15.6">
       <c r="A7" s="10" t="s">
         <v>75</v>
       </c>
@@ -4317,7 +4244,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75">
+    <row r="8" spans="1:9" ht="15.6">
       <c r="A8" s="16" t="s">
         <v>77</v>
       </c>
@@ -4342,7 +4269,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75">
+    <row r="9" spans="1:9" ht="15.6">
       <c r="A9" s="10" t="s">
         <v>78</v>
       </c>
@@ -4367,7 +4294,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75">
+    <row r="10" spans="1:9" ht="15.6">
       <c r="A10" s="16" t="s">
         <v>79</v>
       </c>
@@ -4388,7 +4315,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75">
+    <row r="11" spans="1:9" ht="15.6">
       <c r="A11" s="11" t="s">
         <v>82</v>
       </c>
@@ -4413,7 +4340,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75">
+    <row r="12" spans="1:9" ht="15.6">
       <c r="A12" s="11"/>
       <c r="B12" s="10"/>
       <c r="C12" s="11"/>
@@ -4427,7 +4354,7 @@
       <c r="G12" s="34"/>
       <c r="H12" s="34"/>
     </row>
-    <row r="13" spans="1:9" ht="15.75">
+    <row r="13" spans="1:9" ht="15.6">
       <c r="A13" s="11" t="s">
         <v>83</v>
       </c>
@@ -4450,7 +4377,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.75">
+    <row r="14" spans="1:9" ht="15.6">
       <c r="A14" s="1"/>
       <c r="B14" s="12"/>
       <c r="C14" s="11"/>
@@ -4464,7 +4391,7 @@
       <c r="G14" s="34"/>
       <c r="H14" s="34"/>
     </row>
-    <row r="15" spans="1:9" ht="15.75">
+    <row r="15" spans="1:9" ht="15.6">
       <c r="A15" s="1" t="s">
         <v>85</v>
       </c>
@@ -4487,7 +4414,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.75">
+    <row r="16" spans="1:9" ht="15.6">
       <c r="A16" s="34"/>
       <c r="B16" s="10"/>
       <c r="C16" s="11"/>
@@ -4501,7 +4428,7 @@
       <c r="G16" s="34"/>
       <c r="H16" s="34"/>
     </row>
-    <row r="17" spans="1:9" ht="15.75">
+    <row r="17" spans="1:9" ht="15.6">
       <c r="A17" s="2" t="s">
         <v>86</v>
       </c>
@@ -4526,7 +4453,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15.75">
+    <row r="18" spans="1:9" ht="15.6">
       <c r="A18" s="2"/>
       <c r="B18" s="12"/>
       <c r="C18" s="11"/>
@@ -4540,7 +4467,7 @@
       <c r="G18" s="34"/>
       <c r="H18" s="34"/>
     </row>
-    <row r="19" spans="1:9" ht="15.75">
+    <row r="19" spans="1:9" ht="15.6">
       <c r="A19" s="10" t="s">
         <v>88</v>
       </c>
@@ -4565,7 +4492,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="15.75">
+    <row r="20" spans="1:9" ht="15.6">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -4579,7 +4506,7 @@
       <c r="G20" s="34"/>
       <c r="H20" s="34"/>
     </row>
-    <row r="21" spans="1:9" ht="15.75">
+    <row r="21" spans="1:9" ht="15.6">
       <c r="A21" s="16" t="s">
         <v>89</v>
       </c>
@@ -4604,7 +4531,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.75">
+    <row r="22" spans="1:9" ht="15.6">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -4618,7 +4545,7 @@
       <c r="G22" s="34"/>
       <c r="H22" s="34"/>
     </row>
-    <row r="23" spans="1:9" ht="15.75">
+    <row r="23" spans="1:9" ht="15.6">
       <c r="A23" s="16" t="s">
         <v>90</v>
       </c>
@@ -4643,7 +4570,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.75">
+    <row r="24" spans="1:9" ht="15.6">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
@@ -4657,7 +4584,7 @@
       <c r="G24" s="34"/>
       <c r="H24" s="34"/>
     </row>
-    <row r="25" spans="1:9" ht="15.75">
+    <row r="25" spans="1:9" ht="15.6">
       <c r="A25" s="16" t="s">
         <v>91</v>
       </c>
@@ -4682,7 +4609,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="15.75">
+    <row r="26" spans="1:9" ht="15.6">
       <c r="A26" s="10"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -4696,7 +4623,7 @@
       <c r="G26" s="34"/>
       <c r="H26" s="34"/>
     </row>
-    <row r="27" spans="1:9" ht="15.75">
+    <row r="27" spans="1:9" ht="15.6">
       <c r="A27" s="16" t="s">
         <v>92</v>
       </c>
@@ -4715,7 +4642,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15.75">
+    <row r="28" spans="1:9" ht="15.6">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -4725,7 +4652,7 @@
       <c r="G28" s="34"/>
       <c r="H28" s="34"/>
     </row>
-    <row r="29" spans="1:9" ht="15.75">
+    <row r="29" spans="1:9" ht="15.6">
       <c r="A29" s="16" t="s">
         <v>93</v>
       </c>
@@ -4750,7 +4677,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15.75">
+    <row r="30" spans="1:9" ht="15.6">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -4764,7 +4691,7 @@
       <c r="G30" s="34"/>
       <c r="H30" s="34"/>
     </row>
-    <row r="31" spans="1:9" ht="15.75">
+    <row r="31" spans="1:9" ht="15.6">
       <c r="A31" s="16" t="s">
         <v>94</v>
       </c>
@@ -4789,7 +4716,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15.75">
+    <row r="32" spans="1:9" ht="15.6">
       <c r="A32" s="10"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
@@ -4803,7 +4730,7 @@
       <c r="G32" s="34"/>
       <c r="H32" s="34"/>
     </row>
-    <row r="33" spans="1:9" ht="15.75">
+    <row r="33" spans="1:9" ht="15.6">
       <c r="A33" s="16" t="s">
         <v>95</v>
       </c>
@@ -4828,7 +4755,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.75">
+    <row r="34" spans="1:9" ht="15.6">
       <c r="A34" s="10"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
@@ -4871,12 +4798,12 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FFD4A1B-09FC-41AF-A94F-E802F09E59F5}">
   <dimension ref="A1:I56"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" thickBot="1">
+    <row r="1" spans="1:9" ht="31.9" thickBot="1">
       <c r="A1" s="31" t="s">
         <v>1</v>
       </c>
@@ -4886,22 +4813,22 @@
       <c r="C1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="67" t="s">
+      <c r="D1" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="68"/>
+      <c r="E1" s="69"/>
       <c r="F1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="69" t="s">
+      <c r="G1" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="70"/>
+      <c r="H1" s="71"/>
       <c r="I1" s="36" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75">
+    <row r="2" spans="1:9" ht="15.6">
       <c r="A2" s="16" t="s">
         <v>99</v>
       </c>
@@ -4922,7 +4849,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75">
+    <row r="3" spans="1:9" ht="15.6">
       <c r="A3" s="16"/>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
@@ -4932,7 +4859,7 @@
       <c r="G3" s="17"/>
       <c r="H3" s="18"/>
     </row>
-    <row r="4" spans="1:9" ht="15.75">
+    <row r="4" spans="1:9" ht="15.6">
       <c r="A4" s="10" t="s">
         <v>100</v>
       </c>
@@ -4957,7 +4884,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75">
+    <row r="5" spans="1:9" ht="15.6">
       <c r="A5" s="16"/>
       <c r="B5" s="26"/>
       <c r="C5" s="2"/>
@@ -4971,7 +4898,7 @@
       <c r="G5" s="17"/>
       <c r="H5" s="18"/>
     </row>
-    <row r="6" spans="1:9" ht="15.75">
+    <row r="6" spans="1:9" ht="15.6">
       <c r="A6" s="16"/>
       <c r="B6" s="26"/>
       <c r="C6" s="2"/>
@@ -4981,7 +4908,7 @@
       <c r="G6" s="17"/>
       <c r="H6" s="18"/>
     </row>
-    <row r="7" spans="1:9" ht="15.75">
+    <row r="7" spans="1:9" ht="15.6">
       <c r="A7" s="16" t="s">
         <v>101</v>
       </c>
@@ -5006,7 +4933,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75">
+    <row r="8" spans="1:9" ht="15.6">
       <c r="A8" s="10"/>
       <c r="B8" s="25"/>
       <c r="C8" s="2"/>
@@ -5016,7 +4943,7 @@
       <c r="G8" s="7"/>
       <c r="H8" s="8"/>
     </row>
-    <row r="9" spans="1:9" ht="15.75">
+    <row r="9" spans="1:9" ht="15.6">
       <c r="A9" s="16" t="s">
         <v>104</v>
       </c>
@@ -5041,7 +4968,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75">
+    <row r="10" spans="1:9" ht="15.6">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -5051,7 +4978,7 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:9" ht="15.75">
+    <row r="11" spans="1:9" ht="15.6">
       <c r="A11" s="16" t="s">
         <v>106</v>
       </c>
@@ -5076,7 +5003,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15.75">
+    <row r="12" spans="1:9" ht="15.6">
       <c r="A12" s="11"/>
       <c r="B12" s="10"/>
       <c r="C12" s="11"/>
@@ -5086,7 +5013,7 @@
       <c r="G12" s="34"/>
       <c r="H12" s="34"/>
     </row>
-    <row r="13" spans="1:9" ht="15.75">
+    <row r="13" spans="1:9" ht="15.6">
       <c r="A13" s="11" t="s">
         <v>107</v>
       </c>
@@ -5107,7 +5034,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="15.75">
+    <row r="14" spans="1:9" ht="15.6">
       <c r="A14" s="11"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -5117,7 +5044,7 @@
       <c r="G14" s="34"/>
       <c r="H14" s="34"/>
     </row>
-    <row r="15" spans="1:9" ht="15.75">
+    <row r="15" spans="1:9" ht="15.6">
       <c r="A15" s="1" t="s">
         <v>108</v>
       </c>
@@ -5142,7 +5069,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15.75">
+    <row r="16" spans="1:9" ht="15.6">
       <c r="A16" s="1"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -5156,7 +5083,7 @@
       <c r="G16" s="34"/>
       <c r="H16" s="34"/>
     </row>
-    <row r="17" spans="1:9" ht="15.75">
+    <row r="17" spans="1:9" ht="15.6">
       <c r="A17" s="34"/>
       <c r="B17" s="10"/>
       <c r="C17" s="11"/>
@@ -5170,7 +5097,7 @@
       <c r="G17" s="34"/>
       <c r="H17" s="34"/>
     </row>
-    <row r="18" spans="1:9" ht="15.75">
+    <row r="18" spans="1:9" ht="15.6">
       <c r="A18" s="2"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -5180,7 +5107,7 @@
       <c r="G18" s="34"/>
       <c r="H18" s="34"/>
     </row>
-    <row r="19" spans="1:9" ht="15.75">
+    <row r="19" spans="1:9" ht="15.6">
       <c r="A19" s="2" t="s">
         <v>109</v>
       </c>
@@ -5205,7 +5132,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="15.75">
+    <row r="20" spans="1:9" ht="15.6">
       <c r="A20" s="10"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
@@ -5219,7 +5146,7 @@
       <c r="G20" s="34"/>
       <c r="H20" s="34"/>
     </row>
-    <row r="21" spans="1:9" ht="15.75">
+    <row r="21" spans="1:9" ht="15.6">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -5233,7 +5160,7 @@
       <c r="G21" s="34"/>
       <c r="H21" s="34"/>
     </row>
-    <row r="22" spans="1:9" ht="15.75">
+    <row r="22" spans="1:9" ht="15.6">
       <c r="A22" s="16"/>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
@@ -5243,7 +5170,7 @@
       <c r="G22" s="34"/>
       <c r="H22" s="34"/>
     </row>
-    <row r="23" spans="1:9" ht="15.75">
+    <row r="23" spans="1:9" ht="15.6">
       <c r="A23" s="10" t="s">
         <v>111</v>
       </c>
@@ -5268,7 +5195,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.75">
+    <row r="24" spans="1:9" ht="15.6">
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
       <c r="C24" s="16"/>
@@ -5282,7 +5209,7 @@
       <c r="G24" s="34"/>
       <c r="H24" s="34"/>
     </row>
-    <row r="25" spans="1:9" ht="15.75">
+    <row r="25" spans="1:9" ht="15.6">
       <c r="A25" s="10"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
@@ -5292,7 +5219,7 @@
       <c r="G25" s="34"/>
       <c r="H25" s="34"/>
     </row>
-    <row r="26" spans="1:9" ht="15.75">
+    <row r="26" spans="1:9" ht="15.6">
       <c r="A26" s="16" t="s">
         <v>112</v>
       </c>
@@ -5317,7 +5244,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="15.75">
+    <row r="27" spans="1:9" ht="15.6">
       <c r="A27" s="10"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
@@ -5327,7 +5254,7 @@
       <c r="G27" s="34"/>
       <c r="H27" s="34"/>
     </row>
-    <row r="28" spans="1:9" ht="15.75">
+    <row r="28" spans="1:9" ht="15.6">
       <c r="A28" s="16" t="s">
         <v>113</v>
       </c>
@@ -5352,7 +5279,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15.75">
+    <row r="29" spans="1:9" ht="15.6">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
@@ -5366,7 +5293,7 @@
       <c r="G29" s="34"/>
       <c r="H29" s="34"/>
     </row>
-    <row r="30" spans="1:9" ht="15.75">
+    <row r="30" spans="1:9" ht="15.6">
       <c r="A30" s="16"/>
       <c r="B30" s="16"/>
       <c r="C30" s="16"/>
@@ -5376,7 +5303,7 @@
       <c r="G30" s="34"/>
       <c r="H30" s="34"/>
     </row>
-    <row r="31" spans="1:9" ht="15.75">
+    <row r="31" spans="1:9" ht="15.6">
       <c r="A31" s="10" t="s">
         <v>114</v>
       </c>
@@ -5397,7 +5324,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15.75">
+    <row r="32" spans="1:9" ht="15.6">
       <c r="A32" s="16"/>
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
@@ -5407,7 +5334,7 @@
       <c r="G32" s="34"/>
       <c r="H32" s="34"/>
     </row>
-    <row r="33" spans="1:9" ht="15.75">
+    <row r="33" spans="1:9" ht="15.6">
       <c r="A33" s="10" t="s">
         <v>115</v>
       </c>
@@ -5428,7 +5355,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15.75">
+    <row r="34" spans="1:9" ht="15.6">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -5438,7 +5365,7 @@
       <c r="G34" s="34"/>
       <c r="H34" s="34"/>
     </row>
-    <row r="35" spans="1:9" ht="15.75">
+    <row r="35" spans="1:9" ht="15.6">
       <c r="A35" s="2" t="s">
         <v>116</v>
       </c>
@@ -5463,7 +5390,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="15.75">
+    <row r="36" spans="1:9" ht="15.6">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -5477,7 +5404,7 @@
       <c r="G36" s="34"/>
       <c r="H36" s="34"/>
     </row>
-    <row r="37" spans="1:9" ht="15.75">
+    <row r="37" spans="1:9" ht="15.6">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -5487,7 +5414,7 @@
       <c r="G37" s="34"/>
       <c r="H37" s="34"/>
     </row>
-    <row r="38" spans="1:9" ht="15.75">
+    <row r="38" spans="1:9" ht="15.6">
       <c r="A38" s="2" t="s">
         <v>117</v>
       </c>
@@ -5512,7 +5439,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15.75">
+    <row r="39" spans="1:9" ht="15.6">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -5526,7 +5453,7 @@
       <c r="G39" s="34"/>
       <c r="H39" s="34"/>
     </row>
-    <row r="40" spans="1:9" ht="15.75">
+    <row r="40" spans="1:9" ht="15.6">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -5536,7 +5463,7 @@
       <c r="G40" s="34"/>
       <c r="H40" s="34"/>
     </row>
-    <row r="41" spans="1:9" ht="15.75">
+    <row r="41" spans="1:9" ht="15.6">
       <c r="A41" s="2" t="s">
         <v>118</v>
       </c>
@@ -5557,7 +5484,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="15.75">
+    <row r="42" spans="1:9" ht="15.6">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -5567,7 +5494,7 @@
       <c r="G42" s="34"/>
       <c r="H42" s="34"/>
     </row>
-    <row r="43" spans="1:9" ht="15.75">
+    <row r="43" spans="1:9" ht="15.6">
       <c r="A43" s="2" t="s">
         <v>119</v>
       </c>
@@ -5586,7 +5513,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="15.75">
+    <row r="44" spans="1:9" ht="15.6">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -5596,7 +5523,7 @@
       <c r="G44" s="34"/>
       <c r="H44" s="34"/>
     </row>
-    <row r="45" spans="1:9" ht="15.75">
+    <row r="45" spans="1:9" ht="15.6">
       <c r="A45" s="2" t="s">
         <v>121</v>
       </c>
@@ -5621,7 +5548,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="15.75">
+    <row r="46" spans="1:9" ht="15.6">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -5631,7 +5558,7 @@
       <c r="G46" s="34"/>
       <c r="H46" s="34"/>
     </row>
-    <row r="47" spans="1:9" ht="15.75">
+    <row r="47" spans="1:9" ht="15.6">
       <c r="A47" s="2" t="s">
         <v>122</v>
       </c>
@@ -5654,7 +5581,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="15.75">
+    <row r="48" spans="1:9" ht="15.6">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -5664,7 +5591,7 @@
       <c r="G48" s="34"/>
       <c r="H48" s="34"/>
     </row>
-    <row r="49" spans="1:9" ht="15.75">
+    <row r="49" spans="1:9" ht="15.6">
       <c r="A49" s="2" t="s">
         <v>123</v>
       </c>
@@ -5687,7 +5614,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="15.75">
+    <row r="50" spans="1:9" ht="15.6">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -5703,7 +5630,7 @@
       <c r="G50" s="34"/>
       <c r="H50" s="34"/>
     </row>
-    <row r="51" spans="1:9" ht="15.75">
+    <row r="51" spans="1:9" ht="15.6">
       <c r="A51" s="2" t="s">
         <v>124</v>
       </c>
@@ -5722,7 +5649,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="15.75">
+    <row r="52" spans="1:9" ht="15.6">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -5732,7 +5659,7 @@
       <c r="G52" s="34"/>
       <c r="H52" s="34"/>
     </row>
-    <row r="53" spans="1:9" ht="15.75">
+    <row r="53" spans="1:9" ht="15.6">
       <c r="A53" s="2" t="s">
         <v>124</v>
       </c>
@@ -5751,7 +5678,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="15.75">
+    <row r="54" spans="1:9" ht="15.6">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -5803,729 +5730,619 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0936F1B7-DCFE-4D1A-8448-CC75C7237280}">
-  <dimension ref="A1:M56"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="A1:F56"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="32.25" thickBot="1">
+    <row r="1" spans="1:6" ht="31.15">
       <c r="A1" s="49" t="s">
-        <v>1</v>
+        <v>127</v>
       </c>
       <c r="B1" s="49" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C1" s="49" t="s">
+        <v>129</v>
+      </c>
+      <c r="D1" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="E1" s="50" t="s">
+        <v>131</v>
+      </c>
+      <c r="F1" s="58" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.6">
+      <c r="A2" s="59">
+        <v>45931</v>
+      </c>
+      <c r="B2" s="59">
+        <v>45932</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D2" s="48" t="s">
+        <v>132</v>
+      </c>
+      <c r="E2" s="2">
+        <v>16</v>
+      </c>
+      <c r="F2" s="34" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.6">
+      <c r="A3" s="59">
+        <v>45953</v>
+      </c>
+      <c r="B3" s="59">
+        <v>45954</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D3" s="48" t="s">
+        <v>133</v>
+      </c>
+      <c r="E3" s="2">
+        <v>9</v>
+      </c>
+      <c r="F3" s="34" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.6">
+      <c r="A4" s="59">
+        <v>45953</v>
+      </c>
+      <c r="B4" s="59">
+        <v>45954</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="62">
+        <v>2</v>
+      </c>
+      <c r="F4" s="34" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.6">
+      <c r="A5" s="59">
+        <v>45981</v>
+      </c>
+      <c r="B5" s="59">
+        <v>45982</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="48" t="s">
+        <v>133</v>
+      </c>
+      <c r="E5" s="2">
+        <v>12</v>
+      </c>
+      <c r="F5" s="34" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.6">
+      <c r="A6" s="59">
+        <v>45981</v>
+      </c>
+      <c r="B6" s="59">
+        <v>45982</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1</v>
+      </c>
+      <c r="F6" s="34" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.6">
+      <c r="A7" s="59">
+        <v>45981</v>
+      </c>
+      <c r="B7" s="59">
+        <v>45982</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="2">
         <v>3</v>
       </c>
-      <c r="D1" s="71" t="s">
+      <c r="F7" s="34" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.6">
+      <c r="A8" s="59">
+        <v>45986</v>
+      </c>
+      <c r="B8" s="59">
+        <v>45987</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" s="48" t="s">
+        <v>134</v>
+      </c>
+      <c r="E8" s="2">
+        <v>13</v>
+      </c>
+      <c r="F8" s="34" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.6">
+      <c r="A9" s="59">
+        <v>45986</v>
+      </c>
+      <c r="B9" s="59">
+        <v>45987</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="48" t="s">
+        <v>134</v>
+      </c>
+      <c r="E9" s="2">
+        <v>12</v>
+      </c>
+      <c r="F9" s="34" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.6">
+      <c r="A10" s="59">
+        <v>45995</v>
+      </c>
+      <c r="B10" s="59">
+        <v>45996</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="48" t="s">
+        <v>133</v>
+      </c>
+      <c r="E10" s="2">
+        <v>8</v>
+      </c>
+      <c r="F10" s="34" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.6">
+      <c r="A11" s="59">
+        <v>45995</v>
+      </c>
+      <c r="B11" s="59">
+        <v>45996</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="2">
+        <v>1</v>
+      </c>
+      <c r="F11" s="34" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.6">
+      <c r="A12" s="59">
+        <v>45995</v>
+      </c>
+      <c r="B12" s="59">
+        <v>45996</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="61" t="s">
+        <v>135</v>
+      </c>
+      <c r="E12" s="2">
         <v>4</v>
       </c>
-      <c r="E1" s="72"/>
-      <c r="F1" s="50" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="73" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="74"/>
-      <c r="I1" s="60" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="15.75">
-      <c r="A2" s="51" t="s">
-        <v>128</v>
-      </c>
-      <c r="B2" s="52" t="s">
+      <c r="F12" s="34" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.6">
+      <c r="A13" s="60">
+        <v>46001</v>
+      </c>
+      <c r="B13" s="60">
+        <v>46002</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52" t="s">
-        <v>129</v>
-      </c>
-      <c r="E2" s="53">
-        <v>16</v>
-      </c>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="54" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="15.75">
-      <c r="A3" s="7"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="55"/>
-    </row>
-    <row r="4" spans="1:13" ht="15.75">
-      <c r="A4" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C4" s="2">
-        <v>9</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E4" s="2">
-        <v>2</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="55" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="16.5" thickBot="1">
-      <c r="A5" s="7"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="55"/>
-    </row>
-    <row r="6" spans="1:13" ht="15.75">
-      <c r="A6" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" s="2">
-        <v>12</v>
-      </c>
-      <c r="D6" s="48" t="s">
-        <v>51</v>
-      </c>
-      <c r="E6" s="38">
-        <v>1</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="55" t="s">
-        <v>98</v>
-      </c>
-      <c r="M6" s="61"/>
-    </row>
-    <row r="7" spans="1:13" ht="15.75">
-      <c r="A7" s="7"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E7" s="38">
-        <v>3</v>
-      </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="55"/>
-    </row>
-    <row r="8" spans="1:13" ht="15.75">
-      <c r="A8" s="7"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="55"/>
-    </row>
-    <row r="9" spans="1:13" ht="15.75">
-      <c r="A9" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E9" s="38">
+      <c r="D13" s="61" t="s">
+        <v>133</v>
+      </c>
+      <c r="E13" s="2">
         <v>13</v>
       </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="55" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="15.75">
-      <c r="A10" s="7"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="55"/>
-    </row>
-    <row r="11" spans="1:13" ht="15.75">
-      <c r="A11" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E11" s="38">
-        <v>12</v>
-      </c>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="55" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="15.75">
-      <c r="A12" s="9"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="55"/>
-    </row>
-    <row r="13" spans="1:13" ht="15.75">
-      <c r="A13" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="1">
-        <v>8</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E13" s="2">
-        <v>1</v>
-      </c>
-      <c r="F13" s="2">
-        <v>4</v>
-      </c>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="55" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="15.75">
-      <c r="A14" s="9"/>
-      <c r="B14" s="2"/>
+      <c r="F13" s="34" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.6">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="34"/>
-      <c r="I14" s="55"/>
-    </row>
-    <row r="15" spans="1:13" ht="15.75">
-      <c r="A15" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C15" s="1">
-        <v>13</v>
-      </c>
-      <c r="D15" s="2"/>
+      <c r="F14" s="34"/>
+    </row>
+    <row r="15" spans="1:6" ht="15.6">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="1"/>
       <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="55" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="15.75">
+      <c r="F15" s="34"/>
+    </row>
+    <row r="16" spans="1:6" ht="15.6">
       <c r="A16" s="9"/>
-      <c r="B16" s="2"/>
+      <c r="B16" s="43"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-      <c r="I16" s="55"/>
-    </row>
-    <row r="17" spans="1:9" ht="15.75">
-      <c r="A17" s="56"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
+      <c r="F16" s="51"/>
+    </row>
+    <row r="17" spans="1:6" ht="15.6">
+      <c r="A17" s="52"/>
+      <c r="B17" s="56"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="1"/>
       <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="55"/>
-    </row>
-    <row r="18" spans="1:9" ht="15.75">
+      <c r="F17" s="51"/>
+    </row>
+    <row r="18" spans="1:6" ht="15.6">
       <c r="A18" s="7"/>
-      <c r="B18" s="2"/>
+      <c r="B18" s="41"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="34"/>
-      <c r="I18" s="55"/>
-    </row>
-    <row r="19" spans="1:9" ht="15.75">
+      <c r="F18" s="51"/>
+    </row>
+    <row r="19" spans="1:6" ht="15.6">
       <c r="A19" s="7"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="1"/>
+      <c r="B19" s="41"/>
+      <c r="C19" s="2"/>
       <c r="D19" s="1"/>
       <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="55"/>
-    </row>
-    <row r="20" spans="1:9" ht="15.75">
+      <c r="F19" s="51"/>
+    </row>
+    <row r="20" spans="1:6" ht="15.6">
       <c r="A20" s="7"/>
-      <c r="B20" s="2"/>
+      <c r="B20" s="41"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="34"/>
-      <c r="I20" s="55"/>
-    </row>
-    <row r="21" spans="1:9" ht="15.75">
+      <c r="F20" s="51"/>
+    </row>
+    <row r="21" spans="1:6" ht="15.6">
       <c r="A21" s="7"/>
-      <c r="B21" s="2"/>
+      <c r="B21" s="41"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="55"/>
-    </row>
-    <row r="22" spans="1:9" ht="15.75">
+      <c r="F21" s="51"/>
+    </row>
+    <row r="22" spans="1:6" ht="15.6">
       <c r="A22" s="7"/>
-      <c r="B22" s="2"/>
+      <c r="B22" s="41"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="55"/>
-    </row>
-    <row r="23" spans="1:9" ht="15.75">
+      <c r="E22" s="2"/>
+      <c r="F22" s="51"/>
+    </row>
+    <row r="23" spans="1:6" ht="15.6">
       <c r="A23" s="7"/>
-      <c r="B23" s="2"/>
+      <c r="B23" s="41"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="55"/>
-    </row>
-    <row r="24" spans="1:9" ht="15.75">
+      <c r="F23" s="51"/>
+    </row>
+    <row r="24" spans="1:6" ht="15.6">
       <c r="A24" s="7"/>
-      <c r="B24" s="2"/>
+      <c r="B24" s="41"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="55"/>
-    </row>
-    <row r="25" spans="1:9" ht="15.75">
+      <c r="E24" s="2"/>
+      <c r="F24" s="51"/>
+    </row>
+    <row r="25" spans="1:6" ht="15.6">
       <c r="A25" s="7"/>
-      <c r="B25" s="2"/>
+      <c r="B25" s="41"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="34"/>
-      <c r="I25" s="55"/>
-    </row>
-    <row r="26" spans="1:9" ht="15.75">
+      <c r="F25" s="51"/>
+    </row>
+    <row r="26" spans="1:6" ht="15.6">
       <c r="A26" s="7"/>
-      <c r="B26" s="2"/>
+      <c r="B26" s="41"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="55"/>
-    </row>
-    <row r="27" spans="1:9" ht="15.75">
+      <c r="E26" s="2"/>
+      <c r="F26" s="51"/>
+    </row>
+    <row r="27" spans="1:6" ht="15.6">
       <c r="A27" s="7"/>
-      <c r="B27" s="2"/>
+      <c r="B27" s="41"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="34"/>
-      <c r="I27" s="55"/>
-    </row>
-    <row r="28" spans="1:9" ht="15.75">
+      <c r="F27" s="51"/>
+    </row>
+    <row r="28" spans="1:6" ht="15.6">
       <c r="A28" s="7"/>
-      <c r="B28" s="2"/>
+      <c r="B28" s="41"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="34"/>
-      <c r="H28" s="34"/>
-      <c r="I28" s="55"/>
-    </row>
-    <row r="29" spans="1:9" ht="15.75">
+      <c r="E28" s="2"/>
+      <c r="F28" s="51"/>
+    </row>
+    <row r="29" spans="1:6" ht="15.6">
       <c r="A29" s="7"/>
-      <c r="B29" s="2"/>
+      <c r="B29" s="41"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="34"/>
-      <c r="I29" s="55"/>
-    </row>
-    <row r="30" spans="1:9" ht="15.75">
+      <c r="F29" s="51"/>
+    </row>
+    <row r="30" spans="1:6" ht="15.6">
       <c r="A30" s="7"/>
-      <c r="B30" s="2"/>
+      <c r="B30" s="41"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="34"/>
-      <c r="H30" s="34"/>
-      <c r="I30" s="55"/>
-    </row>
-    <row r="31" spans="1:9" ht="15.75">
+      <c r="E30" s="2"/>
+      <c r="F30" s="51"/>
+    </row>
+    <row r="31" spans="1:6" ht="15.6">
       <c r="A31" s="7"/>
-      <c r="B31" s="2"/>
+      <c r="B31" s="41"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="34"/>
-      <c r="I31" s="55"/>
-    </row>
-    <row r="32" spans="1:9" ht="15.75">
+      <c r="F31" s="51"/>
+    </row>
+    <row r="32" spans="1:6" ht="15.6">
       <c r="A32" s="7"/>
-      <c r="B32" s="2"/>
+      <c r="B32" s="41"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="38"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="34"/>
-      <c r="H32" s="34"/>
-      <c r="I32" s="55"/>
-    </row>
-    <row r="33" spans="1:9" ht="15.75">
+      <c r="E32" s="2"/>
+      <c r="F32" s="51"/>
+    </row>
+    <row r="33" spans="1:6" ht="15.6">
       <c r="A33" s="7"/>
-      <c r="B33" s="2"/>
+      <c r="B33" s="41"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="34"/>
-      <c r="H33" s="34"/>
-      <c r="I33" s="55"/>
-    </row>
-    <row r="34" spans="1:9" ht="15.75">
+      <c r="F33" s="51"/>
+    </row>
+    <row r="34" spans="1:6" ht="15.6">
       <c r="A34" s="7"/>
-      <c r="B34" s="2"/>
+      <c r="B34" s="41"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="34"/>
-      <c r="H34" s="34"/>
-      <c r="I34" s="55"/>
-    </row>
-    <row r="35" spans="1:9" ht="15.75">
+      <c r="F34" s="51"/>
+    </row>
+    <row r="35" spans="1:6" ht="15.6">
       <c r="A35" s="7"/>
-      <c r="B35" s="2"/>
+      <c r="B35" s="41"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="34"/>
-      <c r="I35" s="55"/>
-    </row>
-    <row r="36" spans="1:9" ht="15.75">
+      <c r="F35" s="51"/>
+    </row>
+    <row r="36" spans="1:6" ht="15.6">
       <c r="A36" s="7"/>
-      <c r="B36" s="2"/>
+      <c r="B36" s="41"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="34"/>
-      <c r="H36" s="34"/>
-      <c r="I36" s="55"/>
-    </row>
-    <row r="37" spans="1:9" ht="15.75">
+      <c r="F36" s="51"/>
+    </row>
+    <row r="37" spans="1:6" ht="15.6">
       <c r="A37" s="7"/>
-      <c r="B37" s="2"/>
+      <c r="B37" s="41"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="34"/>
-      <c r="H37" s="34"/>
-      <c r="I37" s="55"/>
-    </row>
-    <row r="38" spans="1:9" ht="15.75">
+      <c r="F37" s="51"/>
+    </row>
+    <row r="38" spans="1:6" ht="15.6">
       <c r="A38" s="7"/>
-      <c r="B38" s="2"/>
+      <c r="B38" s="41"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="34"/>
-      <c r="H38" s="34"/>
-      <c r="I38" s="55"/>
-    </row>
-    <row r="39" spans="1:9" ht="15.75">
+      <c r="F38" s="51"/>
+    </row>
+    <row r="39" spans="1:6" ht="15.6">
       <c r="A39" s="7"/>
-      <c r="B39" s="2"/>
+      <c r="B39" s="41"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="34"/>
-      <c r="H39" s="34"/>
-      <c r="I39" s="55"/>
-    </row>
-    <row r="40" spans="1:9" ht="15.75">
+      <c r="F39" s="51"/>
+    </row>
+    <row r="40" spans="1:6" ht="15.6">
       <c r="A40" s="7"/>
-      <c r="B40" s="2"/>
+      <c r="B40" s="41"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
-      <c r="E40" s="38"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="34"/>
-      <c r="H40" s="34"/>
-      <c r="I40" s="55"/>
-    </row>
-    <row r="41" spans="1:9" ht="15.75">
+      <c r="E40" s="2"/>
+      <c r="F40" s="51"/>
+    </row>
+    <row r="41" spans="1:6" ht="15.6">
       <c r="A41" s="7"/>
-      <c r="B41" s="2"/>
+      <c r="B41" s="41"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="34"/>
-      <c r="H41" s="34"/>
-      <c r="I41" s="55"/>
-    </row>
-    <row r="42" spans="1:9" ht="15.75">
+      <c r="F41" s="51"/>
+    </row>
+    <row r="42" spans="1:6" ht="15.6">
       <c r="A42" s="7"/>
-      <c r="B42" s="2"/>
+      <c r="B42" s="41"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="34"/>
-      <c r="H42" s="34"/>
-      <c r="I42" s="55"/>
-    </row>
-    <row r="43" spans="1:9" ht="15.75">
+      <c r="F42" s="51"/>
+    </row>
+    <row r="43" spans="1:6" ht="15.6">
       <c r="A43" s="7"/>
-      <c r="B43" s="2"/>
+      <c r="B43" s="41"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="34"/>
-      <c r="H43" s="34"/>
-      <c r="I43" s="55"/>
-    </row>
-    <row r="44" spans="1:9" ht="15.75">
+      <c r="F43" s="51"/>
+    </row>
+    <row r="44" spans="1:6" ht="15.6">
       <c r="A44" s="7"/>
-      <c r="B44" s="2"/>
+      <c r="B44" s="41"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="34"/>
-      <c r="H44" s="34"/>
-      <c r="I44" s="55"/>
-    </row>
-    <row r="45" spans="1:9" ht="15.75">
+      <c r="F44" s="51"/>
+    </row>
+    <row r="45" spans="1:6" ht="15.6">
       <c r="A45" s="7"/>
-      <c r="B45" s="2"/>
+      <c r="B45" s="41"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="34"/>
-      <c r="H45" s="34"/>
-      <c r="I45" s="55"/>
-    </row>
-    <row r="46" spans="1:9" ht="15.75">
+      <c r="F45" s="51"/>
+    </row>
+    <row r="46" spans="1:6" ht="15.6">
       <c r="A46" s="7"/>
-      <c r="B46" s="2"/>
+      <c r="B46" s="41"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="34"/>
-      <c r="H46" s="34"/>
-      <c r="I46" s="55"/>
-    </row>
-    <row r="47" spans="1:9" ht="15.75">
+      <c r="F46" s="51"/>
+    </row>
+    <row r="47" spans="1:6" ht="15.6">
       <c r="A47" s="7"/>
-      <c r="B47" s="2"/>
+      <c r="B47" s="41"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="34"/>
-      <c r="H47" s="34"/>
-      <c r="I47" s="55"/>
-    </row>
-    <row r="48" spans="1:9" ht="15.75">
+      <c r="F47" s="51"/>
+    </row>
+    <row r="48" spans="1:6" ht="15.6">
       <c r="A48" s="7"/>
-      <c r="B48" s="2"/>
+      <c r="B48" s="41"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-      <c r="G48" s="34"/>
-      <c r="H48" s="34"/>
-      <c r="I48" s="55"/>
-    </row>
-    <row r="49" spans="1:9" ht="15.75">
+      <c r="F48" s="51"/>
+    </row>
+    <row r="49" spans="1:6" ht="15.6">
       <c r="A49" s="7"/>
-      <c r="B49" s="2"/>
+      <c r="B49" s="41"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-      <c r="G49" s="34"/>
-      <c r="H49" s="34"/>
-      <c r="I49" s="55"/>
-    </row>
-    <row r="50" spans="1:9" ht="15.75">
+      <c r="F49" s="51"/>
+    </row>
+    <row r="50" spans="1:6" ht="15.6">
       <c r="A50" s="7"/>
-      <c r="B50" s="2"/>
+      <c r="B50" s="41"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="34"/>
-      <c r="H50" s="34"/>
-      <c r="I50" s="55"/>
-    </row>
-    <row r="51" spans="1:9" ht="15.75">
+      <c r="F50" s="51"/>
+    </row>
+    <row r="51" spans="1:6" ht="15.6">
       <c r="A51" s="7"/>
-      <c r="B51" s="2"/>
+      <c r="B51" s="41"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="34"/>
-      <c r="H51" s="34"/>
-      <c r="I51" s="55"/>
-    </row>
-    <row r="52" spans="1:9" ht="15.75">
+      <c r="F51" s="51"/>
+    </row>
+    <row r="52" spans="1:6" ht="15.6">
       <c r="A52" s="7"/>
-      <c r="B52" s="2"/>
+      <c r="B52" s="41"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="34"/>
-      <c r="H52" s="34"/>
-      <c r="I52" s="55"/>
-    </row>
-    <row r="53" spans="1:9" ht="15.75">
+      <c r="F52" s="51"/>
+    </row>
+    <row r="53" spans="1:6" ht="15.6">
       <c r="A53" s="7"/>
-      <c r="B53" s="2"/>
+      <c r="B53" s="41"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="34"/>
-      <c r="H53" s="34"/>
-      <c r="I53" s="55"/>
-    </row>
-    <row r="54" spans="1:9" ht="15.75">
+      <c r="F53" s="51"/>
+    </row>
+    <row r="54" spans="1:6" ht="15.6">
       <c r="A54" s="7"/>
-      <c r="B54" s="2"/>
+      <c r="B54" s="41"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-      <c r="G54" s="34"/>
-      <c r="H54" s="34"/>
-      <c r="I54" s="55"/>
-    </row>
-    <row r="55" spans="1:9">
-      <c r="A55" s="56"/>
-      <c r="B55" s="34"/>
+      <c r="F54" s="51"/>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="52"/>
+      <c r="B55" s="56"/>
       <c r="C55" s="34"/>
       <c r="D55" s="34"/>
       <c r="E55" s="34"/>
-      <c r="F55" s="34"/>
-      <c r="G55" s="34"/>
-      <c r="H55" s="34"/>
-      <c r="I55" s="55"/>
-    </row>
-    <row r="56" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A56" s="57"/>
-      <c r="B56" s="58"/>
-      <c r="C56" s="58"/>
-      <c r="D56" s="58"/>
-      <c r="E56" s="58"/>
-      <c r="F56" s="58"/>
-      <c r="G56" s="58"/>
-      <c r="H56" s="58"/>
-      <c r="I56" s="59"/>
+      <c r="F55" s="51"/>
+    </row>
+    <row r="56" spans="1:6" ht="15" thickBot="1">
+      <c r="A56" s="53"/>
+      <c r="B56" s="57"/>
+      <c r="C56" s="54"/>
+      <c r="D56" s="54"/>
+      <c r="E56" s="54"/>
+      <c r="F56" s="55"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="G1:H1"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6740,13 +6557,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8BA6764D-1793-467C-A372-035C4A569BB4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D52E80B6-E067-4713-B5AB-1911B79F73BD}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8753B0C-474A-4C35-B391-9183CB6967F6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{626FAE87-907D-4787-B5EE-252FE5676D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD806336-86C5-4D24-8672-DBD931C5219B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5028445D-4F93-4C65-9BA3-0D173F035BB2}"/>
 </file>
</xml_diff>